<commit_message>
Split quantity and price into columns in stock table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mp3wof2iwnsjKqWXT9wGnu
</commit_message>
<xml_diff>
--- a/stock/stok_artikuly.xlsx
+++ b/stock/stok_artikuly.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Артикулы" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Артикулы'!$A$1:$B$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Артикулы'!$A$1:$D$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -77,13 +77,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -450,1047 +462,1569 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B86"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Артикул</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Описание</t>
         </is>
       </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Количество, шт</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Цена, руб.</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>СтЛонг1_Бордовый S</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Лонгслив облегающий,цвет бордовый размер S, 33 шт, 350р</t>
-        </is>
+          <t>Лонгслив облегающий,цвет бордовый размер S</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>СтЛонг1_Бордовый L</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Лонгслив облегающий,цвет бордовый размер L, 15 шт, 350р</t>
-        </is>
+          <t>Лонгслив облегающий,цвет бордовый размер L</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>СтЛонг1_Шоколад L</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Лонгслив облегающий шоколад размер L 25 штук 350р</t>
-        </is>
+          <t>Лонгслив облегающий шоколад размер L</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>СтДжинсы1 34(40)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Брюки джинсовые размер 34(40) – 13 шт 900р</t>
-        </is>
+          <t>Брюки джинсовые размер 34(40)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>СтДжинсы1 36(42)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Брюки джинсовые размер 36(42) – 17 шт 900р</t>
-        </is>
+          <t>Брюки джинсовые размер 36(42)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>СтКПБ1_Евро_Белый</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>КПБ цвет белый 48 шт 1000р</t>
-        </is>
+          <t>КПБ цвет белый</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>СтКПБ1_Евро_Зеленый</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>КПБ цвет зелёный 2 шт 1000р</t>
-        </is>
+          <t>КПБ цвет зелёный</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>СтКПБ1_Евро_Бежевый</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>КПБ цвет бежевый 1 штука 1000р</t>
-        </is>
+          <t>КПБ цвет бежевый</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>СтБрюки1_Серый 42-170</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Брюки Сингапур цвет серый размер 42-170 8 шт. 350р</t>
-        </is>
+          <t>Брюки Сингапур цвет серый размер 42-170</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>СтПлатье1_Черный 48</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Платье праздничное чёрный цвет 48 размер 10 шт 900р</t>
-        </is>
+          <t>Платье праздничное чёрный цвет 48 размер</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>СтПлатье1_Черный 46</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Платье праздничное чёрный цвет 46 размер 10 шт 900р</t>
-        </is>
+          <t>Платье праздничное чёрный цвет 46 размер</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>СтПиж1_Цвет S(42)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Пижама с цветочным принтом размер S(42) 25 шт 600р</t>
-        </is>
+          <t>Пижама с цветочным принтом размер S(42)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>600</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>СтПлатье2_Кофейный 56</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Платье Фатима шоп цвет кофейный размер 56 1шт 1200р</t>
-        </is>
+          <t>Платье Фатима шоп цвет кофейный размер 56</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>1200</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Оранж 38-44</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Платье оранжевое шифон размер 38-44 8 шт 400р</t>
-        </is>
+          <t>Платье оранжевое шифон размер 38-44</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Оранж 36-42</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Платье оранжевое шифон размер 36-42 9 шт 400р</t>
-        </is>
+          <t>Платье оранжевое шифон размер 36-42</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Розовый 38-44</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Платье розовое шифон размер 38-44 13 шт 400р</t>
-        </is>
+          <t>Платье розовое шифон размер 38-44</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Розовый 36-42</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Платье розовое шифон размер 36-42 14 шт 400р</t>
-        </is>
+          <t>Платье розовое шифон размер 36-42</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Пудра 38-44</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Платье пудра шифон размер 38-44 10 шт 400р</t>
-        </is>
+          <t>Платье пудра шифон размер 38-44</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Пудра 36-42</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Платье пудра шифон размер 36-42 11 шт 400р</t>
-        </is>
+          <t>Платье пудра шифон размер 36-42</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Сирень 38-44</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Платье сирень шифон размер 38-44 5 шт 400р</t>
-        </is>
+          <t>Платье сирень шифон размер 38-44</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Сирень 38-44</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Платье сирень шифон размер 36-42 5 шт 400р</t>
-        </is>
+          <t>Платье сирень шифон размер 36-42</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Фиолет 38-44</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Платье фиолет шифон размер 38-44 11 шт 400р</t>
-        </is>
+          <t>Платье фиолет шифон размер 38-44</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>СтПлатье3_Фиолет 36-42</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Платье фиолет шифон размер 36-42 9 шт 400р</t>
-        </is>
+          <t>Платье фиолет шифон размер 36-42</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Графит S</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер S 5 шт 700р</t>
-        </is>
+          <t>Костюм лапша цвет графит размер S</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Графит M</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер М 1 шт 700р</t>
-        </is>
+          <t>Костюм лапша цвет графит размер М</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Графит L</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер L 23 шт 700р</t>
-        </is>
+          <t>Костюм лапша цвет графит размер L</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Графит XL</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер ХL 11 шт 700р</t>
-        </is>
+          <t>Костюм лапша цвет графит размер ХL</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Черный M</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет чёрный размер M 21 шт 700р</t>
-        </is>
+          <t>Костюм лапша цвет чёрный размер M</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Черный L</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет чёрный размер L 17 шт 700р</t>
-        </is>
+          <t>Костюм лапша цвет чёрный размер L</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Черный XL</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет чёрный размер XL 33 шт 700р</t>
-        </is>
+          <t>Костюм лапша цвет чёрный размер XL</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>СтКостюм1_Коричневый L</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет коричневый размер L 1 штука 700р</t>
-        </is>
+          <t>Костюм лапша цвет коричневый размер L</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>СтРуб1_Зеленый M</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет зелёный размер М 12шт 500р</t>
-        </is>
+          <t>Рубашка Лён мужская цвет зелёный размер М</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>СтРуб1_Зеленый XL</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет зелёный размер XL 1шт 500р</t>
-        </is>
+          <t>Рубашка Лён мужская цвет зелёный размер XL</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>СтРуб1_Бежевый M</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер М 5шт 500р</t>
-        </is>
+          <t>Рубашка Лён мужская цвет бежевый размер М</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>СтРуб1_Бежевый XL</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер XL 1шт 500р</t>
-        </is>
+          <t>Рубашка Лён мужская цвет бежевый размер XL</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>СтРуб1_Бежевый 2XL</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер 2XL 1шт 500р</t>
-        </is>
+          <t>Рубашка Лён мужская цвет бежевый размер 2XL</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>СтРуб1_Бежевый 3XL</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер 3XL 3шт 500р</t>
-        </is>
+          <t>Рубашка Лён мужская цвет бежевый размер 3XL</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>СтРуб1_Бежевый 4XL</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер 4XL 1шт 500р</t>
-        </is>
+          <t>Рубашка Лён мужская цвет бежевый размер 4XL</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>СтПокрывало1</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Покрывало малыш 10 штук 700р</t>
-        </is>
+          <t>Покрывало малыш</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>700</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>СтПлатье4_Полоска 42</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 42 27 шт 450р</t>
-        </is>
+          <t>Платье полоска размер 42</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>СтПлатье4_Полоска 44</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 44 1шт 450р</t>
-        </is>
+          <t>Платье полоска размер 44</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>СтПлатье4_Полоска 46</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 46 4 шт 450р</t>
-        </is>
+          <t>Платье полоска размер 46</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>СтПлатье4_Полоска 48</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 48 23 шт 450р</t>
-        </is>
+          <t>Платье полоска размер 48</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>СтРуб2_Бежевый 40-48</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет беж размер 40-48 2шт 400р</t>
-        </is>
+          <t>Рубашка Полоска цвет беж размер 40-48</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>СтРуб2_Зеленый 40-48</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет зелёный размер 40-48 1шт 400р</t>
-        </is>
+          <t>Рубашка Полоска цвет зелёный размер 40-48</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>СтРуб3_Синий 40-48</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Клетка цвет синий размер 40-48 1шт 400р</t>
-        </is>
+          <t>Рубашка Клетка цвет синий размер 40-48</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>СтРуб2_Желтый S</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет жёлтый размер S 2 шт 400р</t>
-        </is>
+          <t>Рубашка Полоска цвет жёлтый размер S</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>СтРуб2_Розовый M</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет розовый размер М 1шт 400р</t>
-        </is>
+          <t>Рубашка Полоска цвет розовый размер М</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>СтРуб4_СливМасло S</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Рубашка цвет сливочное масло размер S 1шт 400р</t>
-        </is>
+          <t>Рубашка цвет сливочное масло размер S</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>СтРуб4_Желтый S</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Рубашка цвет желтый размер S 1шт 400р</t>
-        </is>
+          <t>Рубашка цвет желтый размер S</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>СтПлатье5_Леопард 42</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Платье шефон леопард размер 42 и 44 по 1 штуке 400р</t>
-        </is>
+          <t>Платье шефон леопард размер 42</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>СтПлатье5_Леопард 44</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Платье шефон леопард размер 42 и 44 по 1 штуке 400р</t>
-        </is>
+          <t>Платье шефон леопард размер 44</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>СтПлатье6 44</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Платье лапша размер 44 и 46 по 1 шт 350р</t>
-        </is>
+          <t>Платье лапша размер 44</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>СтПлатье6 46</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Платье лапша размер 44 и 46 по 1 шт 350р</t>
-        </is>
+          <t>Платье лапша размер 46</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>СтПлатье7 42</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Платье с накидкой размер 42 1шт 800р</t>
-        </is>
+          <t>Платье с накидкой размер 42</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="6" t="n">
+        <v>800</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>СтПлатье8 S</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Платье вязанное размер S 1 шт 450р</t>
-        </is>
+          <t>Платье вязанное размер S</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>СтПлатье9 56</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Платье элина стайл размер 56 1шт 500р</t>
-        </is>
+          <t>Платье элина стайл размер 56</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>СтКофта1_Черный 48</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Кофта мужская черная с топором размер 48 1шт 500р</t>
-        </is>
+          <t>Кофта мужская черная с топором размер 48</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>СтФутб1_Черный 46</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>футболка чёрная с машиной 46 размер 1шт 250р</t>
-        </is>
+          <t>футболка чёрная с машиной 46 размер</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>СтПиджак1_Красный 42</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Красный пиджак 42 размер 4шт 400р</t>
-        </is>
+          <t>Красный пиджак 42 размер</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>СтЮбка1 44</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Юбка коротка с ремнём 44 размер 1шт 400р</t>
-        </is>
+          <t>Юбка коротка с ремнём 44 размер</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>СтПоло1_Серый S</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Поло женское цвет серый размер S 3шт 350р</t>
-        </is>
+          <t>Поло женское цвет серый размер S</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>СтПоло1_Салатовый S</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Поло женское цвет салатовый размер S 1шт 350р</t>
-        </is>
+          <t>Поло женское цвет салатовый размер S</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>СтШорты1_Синий 44</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Шорты льняные женские цвет синий 44 размер 1шт 250р</t>
-        </is>
+          <t>Шорты льняные женские цвет синий 44 размер</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>СтЮбкаШорты1_Голубой S</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Юбка-шорты цвет голубой размер S 1шт 300р</t>
-        </is>
+          <t>Юбка-шорты цвет голубой размер S</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>СтШорты2_Полоска S</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>шорты женские полоска размер S 1шт 250р</t>
-        </is>
+          <t>шорты женские полоска размер S</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>СтШортыДет1 98</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>шорты детские размер 98 1 пачка(3шт) 300р</t>
-        </is>
+          <t>шорты детские размер 98 (пачка по 3 шт)</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>СтШортыДет1 116</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>шорты детские размер 116 2 упаковки(6шт) 300р</t>
-        </is>
+          <t>шорты детские размер 116 (пачка по 3 шт)</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>СтЛегДет1 110</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские размер 110 1пачка(3шт) 350р</t>
-        </is>
+          <t>легинсы детские размер 110 (пачка по 3 шт)</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>СтЛегДет1 128</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские размер 128 4 пачки(12шт) 350р</t>
-        </is>
+          <t>легинсы детские размер 128 (пачка по 3 шт)</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>СтЛегДет2_Серый 110</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские серый цвет размер 110 6шт 100р</t>
-        </is>
+          <t>легинсы детские серый цвет размер 110</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D72" s="6" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>СтЛегДет2_Серый 116</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет серый размер 116 3шт 100р</t>
-        </is>
+          <t>легинсы детские цвет серый размер 116</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>СтЛегДет2_Серый 128</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет серый размер 128 1шт 100р</t>
-        </is>
+          <t>легинсы детские цвет серый размер 128</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <t>СтЛегДет2_Синий 104</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет синий размер 104 6шт 100р</t>
-        </is>
+          <t>легинсы детские цвет синий размер 104</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>СтЛегДет2_Синий 122</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет синий размер 122 3шт 100р</t>
-        </is>
+          <t>легинсы детские цвет синий размер 122</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>СтПлатье10_Графит 48</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Платье шик цвет графит размер 48 5шт 350р</t>
-        </is>
+          <t>Платье шик цвет графит размер 48</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>350</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>СтТуника1_ГолЦветок 54</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Туника голубой цветок размер 54 2шт 250р</t>
-        </is>
+          <t>Туника голубой цветок размер 54</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>СтПоло2_Бордовый 40-48</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Поло полоска цвет бордовый размер 40-48 1шт 400р</t>
-        </is>
+          <t>Поло полоска цвет бордовый размер 40-48</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>СтЛонг2_Бордовый 42-48</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>лонгслив полоска цвет бордовый размер 42-48 1шт 400р</t>
-        </is>
+          <t>лонгслив полоска цвет бордовый размер 42-48</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>400</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>СтПиджак2_Бежевый 56</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Женский пиджак цвет бежевый размер 56 1шт 500р</t>
-        </is>
+          <t>Женский пиджак цвет бежевый размер 56</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>СтКостюм2_Белый 50-52</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>костюм жатко цвет белый размер 50-52 1шт 500р</t>
-        </is>
+          <t>костюм жатко цвет белый размер 50-52</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>СтЮбка2_Белый 50-54</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>юбка длинная цвет белый размер 50-54 1шт 500р</t>
-        </is>
+          <t>юбка длинная цвет белый размер 50-54</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>СтКостюм3_ЧернБел 50</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>костюм цвет чёрно-белый размер 50 1шт 900р</t>
-        </is>
+          <t>костюм цвет чёрно-белый размер 50</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>СтШтапель1_ЧернБел 50</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>штапель цвет чёрно-белый размер 50 1шт 1300р</t>
-        </is>
+          <t>штапель цвет чёрно-белый размер 50</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>1300</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>СтКостюм4_ЧернБел 50</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>костюм двойка женский цвет чёрно-белый размер 50 1шт 1500р</t>
-        </is>
+          <t>костюм двойка женский цвет чёрно-белый размер 50</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" s="6" t="n">
+        <v>1500</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B86"/>
+  <autoFilter ref="A1:D86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add size column to stock table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mp3wof2iwnsjKqWXT9wGnu
</commit_message>
<xml_diff>
--- a/stock/stok_artikuly.xlsx
+++ b/stock/stok_artikuly.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Артикулы" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Артикулы'!$A$1:$D$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Артикулы'!$A$1:$E$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,13 +462,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,6 +493,11 @@
           <t>Цена, руб.</t>
         </is>
       </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Размер</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -501,7 +507,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Лонгслив облегающий,цвет бордовый размер S</t>
+          <t>Лонгслив облегающий,цвет бордовый</t>
         </is>
       </c>
       <c r="C2" s="5" t="n">
@@ -510,6 +516,11 @@
       <c r="D2" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -519,7 +530,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Лонгслив облегающий,цвет бордовый размер L</t>
+          <t>Лонгслив облегающий,цвет бордовый</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -528,6 +539,11 @@
       <c r="D3" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -537,7 +553,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Лонгслив облегающий шоколад размер L</t>
+          <t>Лонгслив облегающий шоколад</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
@@ -546,6 +562,11 @@
       <c r="D4" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -555,7 +576,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Брюки джинсовые размер 34(40)</t>
+          <t>Брюки джинсовые</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -564,6 +585,11 @@
       <c r="D5" s="6" t="n">
         <v>900</v>
       </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>34(40)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -573,7 +599,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Брюки джинсовые размер 36(42)</t>
+          <t>Брюки джинсовые</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
@@ -582,6 +608,11 @@
       <c r="D6" s="6" t="n">
         <v>900</v>
       </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>36(42)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -600,6 +631,11 @@
       <c r="D7" s="6" t="n">
         <v>1000</v>
       </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Евро</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -618,6 +654,11 @@
       <c r="D8" s="6" t="n">
         <v>1000</v>
       </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Евро</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -636,6 +677,11 @@
       <c r="D9" s="6" t="n">
         <v>1000</v>
       </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Евро</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -645,7 +691,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Брюки Сингапур цвет серый размер 42-170</t>
+          <t>Брюки Сингапур цвет серый</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
@@ -654,6 +700,11 @@
       <c r="D10" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>42-170</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -663,7 +714,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Платье праздничное чёрный цвет 48 размер</t>
+          <t>Платье праздничное чёрный цвет</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
@@ -672,6 +723,11 @@
       <c r="D11" s="6" t="n">
         <v>900</v>
       </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -681,7 +737,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Платье праздничное чёрный цвет 46 размер</t>
+          <t>Платье праздничное чёрный цвет</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
@@ -690,6 +746,11 @@
       <c r="D12" s="6" t="n">
         <v>900</v>
       </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -699,7 +760,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Пижама с цветочным принтом размер S(42)</t>
+          <t>Пижама с цветочным принтом</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
@@ -708,6 +769,11 @@
       <c r="D13" s="6" t="n">
         <v>600</v>
       </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>S(42)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -717,7 +783,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Платье Фатима шоп цвет кофейный размер 56</t>
+          <t>Платье Фатима шоп цвет кофейный</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
@@ -726,6 +792,11 @@
       <c r="D14" s="6" t="n">
         <v>1200</v>
       </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -735,7 +806,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Платье оранжевое шифон размер 38-44</t>
+          <t>Платье оранжевое шифон</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
@@ -744,6 +815,11 @@
       <c r="D15" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>38-44</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -753,7 +829,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Платье оранжевое шифон размер 36-42</t>
+          <t>Платье оранжевое шифон</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -762,6 +838,11 @@
       <c r="D16" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>36-42</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -771,7 +852,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Платье розовое шифон размер 38-44</t>
+          <t>Платье розовое шифон</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
@@ -780,6 +861,11 @@
       <c r="D17" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>38-44</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -789,7 +875,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Платье розовое шифон размер 36-42</t>
+          <t>Платье розовое шифон</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
@@ -798,6 +884,11 @@
       <c r="D18" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>36-42</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -807,7 +898,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Платье пудра шифон размер 38-44</t>
+          <t>Платье пудра шифон</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
@@ -816,6 +907,11 @@
       <c r="D19" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>38-44</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -825,7 +921,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Платье пудра шифон размер 36-42</t>
+          <t>Платье пудра шифон</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
@@ -834,6 +930,11 @@
       <c r="D20" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>36-42</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -843,7 +944,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Платье сирень шифон размер 38-44</t>
+          <t>Платье сирень шифон</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
@@ -852,6 +953,11 @@
       <c r="D21" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>38-44</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -861,7 +967,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Платье сирень шифон размер 36-42</t>
+          <t>Платье сирень шифон</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
@@ -870,6 +976,11 @@
       <c r="D22" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>36-42</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -879,7 +990,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Платье фиолет шифон размер 38-44</t>
+          <t>Платье фиолет шифон</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
@@ -888,6 +999,11 @@
       <c r="D23" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>38-44</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -897,7 +1013,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Платье фиолет шифон размер 36-42</t>
+          <t>Платье фиолет шифон</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
@@ -906,6 +1022,11 @@
       <c r="D24" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>36-42</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -915,7 +1036,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер S</t>
+          <t>Костюм лапша цвет графит</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
@@ -924,6 +1045,11 @@
       <c r="D25" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -933,7 +1059,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер М</t>
+          <t>Костюм лапша цвет графит</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
@@ -942,6 +1068,11 @@
       <c r="D26" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -951,7 +1082,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер L</t>
+          <t>Костюм лапша цвет графит</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
@@ -960,6 +1091,11 @@
       <c r="D27" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -969,7 +1105,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет графит размер ХL</t>
+          <t>Костюм лапша цвет графит</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
@@ -978,6 +1114,11 @@
       <c r="D28" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -987,7 +1128,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет чёрный размер M</t>
+          <t>Костюм лапша цвет чёрный</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -996,6 +1137,11 @@
       <c r="D29" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1005,7 +1151,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет чёрный размер L</t>
+          <t>Костюм лапша цвет чёрный</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
@@ -1014,6 +1160,11 @@
       <c r="D30" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1023,7 +1174,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет чёрный размер XL</t>
+          <t>Костюм лапша цвет чёрный</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
@@ -1032,6 +1183,11 @@
       <c r="D31" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1041,7 +1197,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Костюм лапша цвет коричневый размер L</t>
+          <t>Костюм лапша цвет коричневый</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
@@ -1050,6 +1206,11 @@
       <c r="D32" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1059,7 +1220,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет зелёный размер М</t>
+          <t>Рубашка Лён мужская цвет зелёный</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
@@ -1068,6 +1229,11 @@
       <c r="D33" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1077,7 +1243,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет зелёный размер XL</t>
+          <t>Рубашка Лён мужская цвет зелёный</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -1086,6 +1252,11 @@
       <c r="D34" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1095,7 +1266,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер М</t>
+          <t>Рубашка Лён мужская цвет бежевый</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
@@ -1104,6 +1275,11 @@
       <c r="D35" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1113,7 +1289,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер XL</t>
+          <t>Рубашка Лён мужская цвет бежевый</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
@@ -1122,6 +1298,11 @@
       <c r="D36" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -1131,7 +1312,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер 2XL</t>
+          <t>Рубашка Лён мужская цвет бежевый</t>
         </is>
       </c>
       <c r="C37" s="5" t="n">
@@ -1140,6 +1321,11 @@
       <c r="D37" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>2XL</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -1149,7 +1335,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер 3XL</t>
+          <t>Рубашка Лён мужская цвет бежевый</t>
         </is>
       </c>
       <c r="C38" s="5" t="n">
@@ -1158,6 +1344,11 @@
       <c r="D38" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>3XL</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -1167,7 +1358,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Лён мужская цвет бежевый размер 4XL</t>
+          <t>Рубашка Лён мужская цвет бежевый</t>
         </is>
       </c>
       <c r="C39" s="5" t="n">
@@ -1176,6 +1367,11 @@
       <c r="D39" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>4XL</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1194,6 +1390,7 @@
       <c r="D40" s="6" t="n">
         <v>700</v>
       </c>
+      <c r="E40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -1203,7 +1400,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 42</t>
+          <t>Платье полоска</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
@@ -1212,6 +1409,11 @@
       <c r="D41" s="6" t="n">
         <v>450</v>
       </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -1221,7 +1423,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 44</t>
+          <t>Платье полоска</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
@@ -1230,6 +1432,11 @@
       <c r="D42" s="6" t="n">
         <v>450</v>
       </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -1239,7 +1446,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 46</t>
+          <t>Платье полоска</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
@@ -1248,6 +1455,11 @@
       <c r="D43" s="6" t="n">
         <v>450</v>
       </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -1257,7 +1469,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Платье полоска размер 48</t>
+          <t>Платье полоска</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
@@ -1266,6 +1478,11 @@
       <c r="D44" s="6" t="n">
         <v>450</v>
       </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -1275,7 +1492,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет беж размер 40-48</t>
+          <t>Рубашка Полоска цвет беж</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -1284,6 +1501,11 @@
       <c r="D45" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>40-48</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -1293,7 +1515,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет зелёный размер 40-48</t>
+          <t>Рубашка Полоска цвет зелёный</t>
         </is>
       </c>
       <c r="C46" s="5" t="n">
@@ -1302,6 +1524,11 @@
       <c r="D46" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>40-48</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -1311,7 +1538,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Клетка цвет синий размер 40-48</t>
+          <t>Рубашка Клетка цвет синий</t>
         </is>
       </c>
       <c r="C47" s="5" t="n">
@@ -1320,6 +1547,11 @@
       <c r="D47" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>40-48</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -1329,7 +1561,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет жёлтый размер S</t>
+          <t>Рубашка Полоска цвет жёлтый</t>
         </is>
       </c>
       <c r="C48" s="5" t="n">
@@ -1338,6 +1570,11 @@
       <c r="D48" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -1347,7 +1584,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Рубашка Полоска цвет розовый размер М</t>
+          <t>Рубашка Полоска цвет розовый</t>
         </is>
       </c>
       <c r="C49" s="5" t="n">
@@ -1356,6 +1593,11 @@
       <c r="D49" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -1365,7 +1607,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Рубашка цвет сливочное масло размер S</t>
+          <t>Рубашка цвет сливочное масло</t>
         </is>
       </c>
       <c r="C50" s="5" t="n">
@@ -1374,6 +1616,11 @@
       <c r="D50" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -1383,7 +1630,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Рубашка цвет желтый размер S</t>
+          <t>Рубашка цвет желтый</t>
         </is>
       </c>
       <c r="C51" s="5" t="n">
@@ -1392,6 +1639,11 @@
       <c r="D51" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -1401,7 +1653,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Платье шефон леопард размер 42</t>
+          <t>Платье шефон леопард</t>
         </is>
       </c>
       <c r="C52" s="5" t="n">
@@ -1410,6 +1662,11 @@
       <c r="D52" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -1419,7 +1676,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Платье шефон леопард размер 44</t>
+          <t>Платье шефон леопард</t>
         </is>
       </c>
       <c r="C53" s="5" t="n">
@@ -1428,6 +1685,11 @@
       <c r="D53" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -1437,7 +1699,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Платье лапша размер 44</t>
+          <t>Платье лапша</t>
         </is>
       </c>
       <c r="C54" s="5" t="n">
@@ -1446,6 +1708,11 @@
       <c r="D54" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -1455,7 +1722,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Платье лапша размер 46</t>
+          <t>Платье лапша</t>
         </is>
       </c>
       <c r="C55" s="5" t="n">
@@ -1464,6 +1731,11 @@
       <c r="D55" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -1473,7 +1745,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Платье с накидкой размер 42</t>
+          <t>Платье с накидкой</t>
         </is>
       </c>
       <c r="C56" s="5" t="n">
@@ -1482,6 +1754,11 @@
       <c r="D56" s="6" t="n">
         <v>800</v>
       </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -1491,7 +1768,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Платье вязанное размер S</t>
+          <t>Платье вязанное</t>
         </is>
       </c>
       <c r="C57" s="5" t="n">
@@ -1500,6 +1777,11 @@
       <c r="D57" s="6" t="n">
         <v>450</v>
       </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -1509,7 +1791,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Платье элина стайл размер 56</t>
+          <t>Платье элина стайл</t>
         </is>
       </c>
       <c r="C58" s="5" t="n">
@@ -1518,6 +1800,11 @@
       <c r="D58" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -1527,7 +1814,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Кофта мужская черная с топором размер 48</t>
+          <t>Кофта мужская черная с топором</t>
         </is>
       </c>
       <c r="C59" s="5" t="n">
@@ -1536,6 +1823,11 @@
       <c r="D59" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -1545,7 +1837,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>футболка чёрная с машиной 46 размер</t>
+          <t>футболка чёрная с машиной</t>
         </is>
       </c>
       <c r="C60" s="5" t="n">
@@ -1554,6 +1846,11 @@
       <c r="D60" s="6" t="n">
         <v>250</v>
       </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -1563,7 +1860,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Красный пиджак 42 размер</t>
+          <t>Красный пиджак</t>
         </is>
       </c>
       <c r="C61" s="5" t="n">
@@ -1572,6 +1869,11 @@
       <c r="D61" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -1581,7 +1883,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Юбка коротка с ремнём 44 размер</t>
+          <t>Юбка коротка с ремнём</t>
         </is>
       </c>
       <c r="C62" s="5" t="n">
@@ -1590,6 +1892,11 @@
       <c r="D62" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -1599,7 +1906,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Поло женское цвет серый размер S</t>
+          <t>Поло женское цвет серый</t>
         </is>
       </c>
       <c r="C63" s="5" t="n">
@@ -1608,6 +1915,11 @@
       <c r="D63" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -1617,7 +1929,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Поло женское цвет салатовый размер S</t>
+          <t>Поло женское цвет салатовый</t>
         </is>
       </c>
       <c r="C64" s="5" t="n">
@@ -1626,6 +1938,11 @@
       <c r="D64" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -1635,7 +1952,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Шорты льняные женские цвет синий 44 размер</t>
+          <t>Шорты льняные женские цвет синий</t>
         </is>
       </c>
       <c r="C65" s="5" t="n">
@@ -1644,6 +1961,11 @@
       <c r="D65" s="6" t="n">
         <v>250</v>
       </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -1653,7 +1975,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Юбка-шорты цвет голубой размер S</t>
+          <t>Юбка-шорты цвет голубой</t>
         </is>
       </c>
       <c r="C66" s="5" t="n">
@@ -1662,6 +1984,11 @@
       <c r="D66" s="6" t="n">
         <v>300</v>
       </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -1671,7 +1998,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>шорты женские полоска размер S</t>
+          <t>шорты женские полоска</t>
         </is>
       </c>
       <c r="C67" s="5" t="n">
@@ -1680,6 +2007,11 @@
       <c r="D67" s="6" t="n">
         <v>250</v>
       </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -1689,7 +2021,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>шорты детские размер 98 (пачка по 3 шт)</t>
+          <t>шорты детские (пачка по 3 шт)</t>
         </is>
       </c>
       <c r="C68" s="5" t="n">
@@ -1698,6 +2030,11 @@
       <c r="D68" s="6" t="n">
         <v>300</v>
       </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -1707,7 +2044,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>шорты детские размер 116 (пачка по 3 шт)</t>
+          <t>шорты детские (пачка по 3 шт)</t>
         </is>
       </c>
       <c r="C69" s="5" t="n">
@@ -1716,6 +2053,11 @@
       <c r="D69" s="6" t="n">
         <v>300</v>
       </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -1725,7 +2067,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские размер 110 (пачка по 3 шт)</t>
+          <t>легинсы детские (пачка по 3 шт)</t>
         </is>
       </c>
       <c r="C70" s="5" t="n">
@@ -1734,6 +2076,11 @@
       <c r="D70" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -1743,7 +2090,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские размер 128 (пачка по 3 шт)</t>
+          <t>легинсы детские (пачка по 3 шт)</t>
         </is>
       </c>
       <c r="C71" s="5" t="n">
@@ -1752,6 +2099,11 @@
       <c r="D71" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -1761,7 +2113,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские серый цвет размер 110</t>
+          <t>легинсы детские серый цвет</t>
         </is>
       </c>
       <c r="C72" s="5" t="n">
@@ -1770,6 +2122,11 @@
       <c r="D72" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -1779,7 +2136,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет серый размер 116</t>
+          <t>легинсы детские цвет серый</t>
         </is>
       </c>
       <c r="C73" s="5" t="n">
@@ -1788,6 +2145,11 @@
       <c r="D73" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -1797,7 +2159,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет серый размер 128</t>
+          <t>легинсы детские цвет серый</t>
         </is>
       </c>
       <c r="C74" s="5" t="n">
@@ -1806,6 +2168,11 @@
       <c r="D74" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -1815,7 +2182,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет синий размер 104</t>
+          <t>легинсы детские цвет синий</t>
         </is>
       </c>
       <c r="C75" s="5" t="n">
@@ -1824,6 +2191,11 @@
       <c r="D75" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -1833,7 +2205,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>легинсы детские цвет синий размер 122</t>
+          <t>легинсы детские цвет синий</t>
         </is>
       </c>
       <c r="C76" s="5" t="n">
@@ -1842,6 +2214,11 @@
       <c r="D76" s="6" t="n">
         <v>100</v>
       </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -1851,7 +2228,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Платье шик цвет графит размер 48</t>
+          <t>Платье шик цвет графит</t>
         </is>
       </c>
       <c r="C77" s="5" t="n">
@@ -1860,6 +2237,11 @@
       <c r="D77" s="6" t="n">
         <v>350</v>
       </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -1869,7 +2251,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Туника голубой цветок размер 54</t>
+          <t>Туника голубой цветок</t>
         </is>
       </c>
       <c r="C78" s="5" t="n">
@@ -1878,6 +2260,11 @@
       <c r="D78" s="6" t="n">
         <v>250</v>
       </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -1887,7 +2274,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Поло полоска цвет бордовый размер 40-48</t>
+          <t>Поло полоска цвет бордовый</t>
         </is>
       </c>
       <c r="C79" s="5" t="n">
@@ -1896,6 +2283,11 @@
       <c r="D79" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>40-48</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -1905,7 +2297,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>лонгслив полоска цвет бордовый размер 42-48</t>
+          <t>лонгслив полоска цвет бордовый</t>
         </is>
       </c>
       <c r="C80" s="5" t="n">
@@ -1914,6 +2306,11 @@
       <c r="D80" s="6" t="n">
         <v>400</v>
       </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>42-48</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -1923,7 +2320,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Женский пиджак цвет бежевый размер 56</t>
+          <t>Женский пиджак цвет бежевый</t>
         </is>
       </c>
       <c r="C81" s="5" t="n">
@@ -1932,6 +2329,11 @@
       <c r="D81" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -1941,7 +2343,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>костюм жатко цвет белый размер 50-52</t>
+          <t>костюм жатко цвет белый</t>
         </is>
       </c>
       <c r="C82" s="5" t="n">
@@ -1950,6 +2352,11 @@
       <c r="D82" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>50-52</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -1959,7 +2366,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>юбка длинная цвет белый размер 50-54</t>
+          <t>юбка длинная цвет белый</t>
         </is>
       </c>
       <c r="C83" s="5" t="n">
@@ -1968,6 +2375,11 @@
       <c r="D83" s="6" t="n">
         <v>500</v>
       </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>50-54</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -1977,7 +2389,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>костюм цвет чёрно-белый размер 50</t>
+          <t>костюм цвет чёрно-белый</t>
         </is>
       </c>
       <c r="C84" s="5" t="n">
@@ -1986,6 +2398,11 @@
       <c r="D84" s="6" t="n">
         <v>900</v>
       </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -1995,7 +2412,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>штапель цвет чёрно-белый размер 50</t>
+          <t>штапель цвет чёрно-белый</t>
         </is>
       </c>
       <c r="C85" s="5" t="n">
@@ -2004,6 +2421,11 @@
       <c r="D85" s="6" t="n">
         <v>1300</v>
       </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -2013,7 +2435,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>костюм двойка женский цвет чёрно-белый размер 50</t>
+          <t>костюм двойка женский цвет чёрно-белый</t>
         </is>
       </c>
       <c r="C86" s="5" t="n">
@@ -2022,9 +2444,14 @@
       <c r="D86" s="6" t="n">
         <v>1500</v>
       </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D86"/>
+  <autoFilter ref="A1:E86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove size from vendor codes in stock table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mp3wof2iwnsjKqWXT9wGnu
</commit_message>
<xml_diff>
--- a/stock/stok_artikuly.xlsx
+++ b/stock/stok_artikuly.xlsx
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>СтЛонг1_Бордовый S</t>
+          <t>СтЛонг1_Бордовый</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>СтЛонг1_Бордовый L</t>
+          <t>СтЛонг1_Бордовый</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -548,7 +548,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>СтЛонг1_Шоколад L</t>
+          <t>СтЛонг1_Шоколад</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -571,7 +571,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>СтДжинсы1 34(40)</t>
+          <t>СтДжинсы1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -594,7 +594,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>СтДжинсы1 36(42)</t>
+          <t>СтДжинсы1</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>СтКПБ1_Евро_Белый</t>
+          <t>СтКПБ1_Белый</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -640,7 +640,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>СтКПБ1_Евро_Зеленый</t>
+          <t>СтКПБ1_Зеленый</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>СтКПБ1_Евро_Бежевый</t>
+          <t>СтКПБ1_Бежевый</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -686,7 +686,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>СтБрюки1_Серый 42-170</t>
+          <t>СтБрюки1_Серый</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -709,7 +709,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье1_Черный 48</t>
+          <t>СтПлатье1_Черный</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -732,7 +732,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье1_Черный 46</t>
+          <t>СтПлатье1_Черный</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>СтПиж1_Цвет S(42)</t>
+          <t>СтПиж1_Цвет</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье2_Кофейный 56</t>
+          <t>СтПлатье2_Кофейный</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -801,7 +801,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Оранж 38-44</t>
+          <t>СтПлатье3_Оранж</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -824,7 +824,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Оранж 36-42</t>
+          <t>СтПлатье3_Оранж</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -847,7 +847,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Розовый 38-44</t>
+          <t>СтПлатье3_Розовый</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -870,7 +870,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Розовый 36-42</t>
+          <t>СтПлатье3_Розовый</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Пудра 38-44</t>
+          <t>СтПлатье3_Пудра</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Пудра 36-42</t>
+          <t>СтПлатье3_Пудра</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -939,7 +939,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Сирень 38-44</t>
+          <t>СтПлатье3_Сирень</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -962,7 +962,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Сирень 38-44</t>
+          <t>СтПлатье3_Сирень</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Фиолет 38-44</t>
+          <t>СтПлатье3_Фиолет</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1008,7 +1008,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье3_Фиолет 36-42</t>
+          <t>СтПлатье3_Фиолет</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1031,7 +1031,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Графит S</t>
+          <t>СтКостюм1_Графит</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1054,7 +1054,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Графит M</t>
+          <t>СтКостюм1_Графит</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1077,7 +1077,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Графит L</t>
+          <t>СтКостюм1_Графит</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1100,7 +1100,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Графит XL</t>
+          <t>СтКостюм1_Графит</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1123,7 +1123,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Черный M</t>
+          <t>СтКостюм1_Черный</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1146,7 +1146,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Черный L</t>
+          <t>СтКостюм1_Черный</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1169,7 +1169,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Черный XL</t>
+          <t>СтКостюм1_Черный</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1192,7 +1192,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм1_Коричневый L</t>
+          <t>СтКостюм1_Коричневый</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>СтРуб1_Зеленый M</t>
+          <t>СтРуб1_Зеленый</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1238,7 +1238,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>СтРуб1_Зеленый XL</t>
+          <t>СтРуб1_Зеленый</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>СтРуб1_Бежевый M</t>
+          <t>СтРуб1_Бежевый</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>СтРуб1_Бежевый XL</t>
+          <t>СтРуб1_Бежевый</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>СтРуб1_Бежевый 2XL</t>
+          <t>СтРуб1_Бежевый</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1330,7 +1330,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>СтРуб1_Бежевый 3XL</t>
+          <t>СтРуб1_Бежевый</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1353,7 +1353,7 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>СтРуб1_Бежевый 4XL</t>
+          <t>СтРуб1_Бежевый</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье4_Полоска 42</t>
+          <t>СтПлатье4_Полоска</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1418,7 +1418,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье4_Полоска 44</t>
+          <t>СтПлатье4_Полоска</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье4_Полоска 46</t>
+          <t>СтПлатье4_Полоска</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -1464,7 +1464,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье4_Полоска 48</t>
+          <t>СтПлатье4_Полоска</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>СтРуб2_Бежевый 40-48</t>
+          <t>СтРуб2_Бежевый</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -1510,7 +1510,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>СтРуб2_Зеленый 40-48</t>
+          <t>СтРуб2_Зеленый</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1533,7 +1533,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>СтРуб3_Синий 40-48</t>
+          <t>СтРуб3_Синий</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -1556,7 +1556,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>СтРуб2_Желтый S</t>
+          <t>СтРуб2_Желтый</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -1579,7 +1579,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>СтРуб2_Розовый M</t>
+          <t>СтРуб2_Розовый</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -1602,7 +1602,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>СтРуб4_СливМасло S</t>
+          <t>СтРуб4_СливМасло</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -1625,7 +1625,7 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>СтРуб4_Желтый S</t>
+          <t>СтРуб4_Желтый</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -1648,7 +1648,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье5_Леопард 42</t>
+          <t>СтПлатье5_Леопард</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -1671,7 +1671,7 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье5_Леопард 44</t>
+          <t>СтПлатье5_Леопард</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье6 44</t>
+          <t>СтПлатье6</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -1717,7 +1717,7 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье6 46</t>
+          <t>СтПлатье6</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье7 42</t>
+          <t>СтПлатье7</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -1763,7 +1763,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье8 S</t>
+          <t>СтПлатье8</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -1786,7 +1786,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье9 56</t>
+          <t>СтПлатье9</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -1809,7 +1809,7 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>СтКофта1_Черный 48</t>
+          <t>СтКофта1_Черный</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -1832,7 +1832,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>СтФутб1_Черный 46</t>
+          <t>СтФутб1_Черный</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -1855,7 +1855,7 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>СтПиджак1_Красный 42</t>
+          <t>СтПиджак1_Красный</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -1878,7 +1878,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>СтЮбка1 44</t>
+          <t>СтЮбка1</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -1901,7 +1901,7 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>СтПоло1_Серый S</t>
+          <t>СтПоло1_Серый</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -1924,7 +1924,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>СтПоло1_Салатовый S</t>
+          <t>СтПоло1_Салатовый</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -1947,7 +1947,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>СтШорты1_Синий 44</t>
+          <t>СтШорты1_Синий</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -1970,7 +1970,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>СтЮбкаШорты1_Голубой S</t>
+          <t>СтЮбкаШорты1_Голубой</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -1993,7 +1993,7 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>СтШорты2_Полоска S</t>
+          <t>СтШорты2_Полоска</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -2016,7 +2016,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>СтШортыДет1 98</t>
+          <t>СтШортыДет1</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -2039,7 +2039,7 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>СтШортыДет1 116</t>
+          <t>СтШортыДет1</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -2062,7 +2062,7 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>СтЛегДет1 110</t>
+          <t>СтЛегДет1</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2085,7 +2085,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>СтЛегДет1 128</t>
+          <t>СтЛегДет1</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -2108,7 +2108,7 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>СтЛегДет2_Серый 110</t>
+          <t>СтЛегДет2_Серый</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>СтЛегДет2_Серый 116</t>
+          <t>СтЛегДет2_Серый</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>СтЛегДет2_Серый 128</t>
+          <t>СтЛегДет2_Серый</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>СтЛегДет2_Синий 104</t>
+          <t>СтЛегДет2_Синий</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -2200,7 +2200,7 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>СтЛегДет2_Синий 122</t>
+          <t>СтЛегДет2_Синий</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -2223,7 +2223,7 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>СтПлатье10_Графит 48</t>
+          <t>СтПлатье10_Графит</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2246,7 +2246,7 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>СтТуника1_ГолЦветок 54</t>
+          <t>СтТуника1_ГолЦветок</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2269,7 +2269,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>СтПоло2_Бордовый 40-48</t>
+          <t>СтПоло2_Бордовый</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -2292,7 +2292,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>СтЛонг2_Бордовый 42-48</t>
+          <t>СтЛонг2_Бордовый</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2315,7 +2315,7 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>СтПиджак2_Бежевый 56</t>
+          <t>СтПиджак2_Бежевый</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -2338,7 +2338,7 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм2_Белый 50-52</t>
+          <t>СтКостюм2_Белый</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -2361,7 +2361,7 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>СтЮбка2_Белый 50-54</t>
+          <t>СтЮбка2_Белый</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -2384,7 +2384,7 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм3_ЧернБел 50</t>
+          <t>СтКостюм3_ЧернБел</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -2407,7 +2407,7 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>СтШтапель1_ЧернБел 50</t>
+          <t>СтШтапель1_ЧернБел</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -2430,7 +2430,7 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>СтКостюм4_ЧернБел 50</t>
+          <t>СтКостюм4_ЧернБел</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">

</xml_diff>